<commit_message>
Fix overlapping/jumbled charts inside the WCC spreadsheet
Native Excel charts were anchored on top of each other and illegible:

- Dashboard: 2x2 chart grid was anchored at B/G with 13cm-wide charts,
  so the left chart overran the right one. Re-anchored left column at B,
  right column at H (clear 7.7cm gap), width 12cm, two row bands at
  rows 15 and 35; footer moved to row 56.
- Budget: pie + bar were both on row 28 side by side and overlapped.
  Now stacked vertically (pie A28, bar A47).
- RSVP: meal bar was anchored at E26, inside the donut's vertical span
  (E15, 8cm tall). Both moved to column H and stacked (H4 + H20) with a
  clear gap, clear of the data tables.

Verified non-overlap via the drawing XML EMU extents.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016YnPMpeJWKT9dx5HR1K2in
</commit_message>
<xml_diff>
--- a/products/wedding-command-center/Wedding_Command_Center.xlsx
+++ b/products/wedding-command-center/Wedding_Command_Center.xlsx
@@ -1430,7 +1430,7 @@
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1447,12 +1447,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>14</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1471,10 +1471,10 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -1491,12 +1491,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>32</row>
+      <row>34</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="4680000" cy="3240000"/>
+    <ext cx="4320000" cy="3060000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1540,12 +1540,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>46</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="3240000"/>
+    <ext cx="6480000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1594,12 +1594,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3960000" cy="2880000"/>
+    <ext cx="4320000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1616,12 +1616,12 @@
   </oneCellAnchor>
   <oneCellAnchor>
     <from>
-      <col>4</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>25</row>
+      <row>19</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="3960000" cy="2880000"/>
+    <ext cx="4320000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1956,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2185,8 +2185,8 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="26" customHeight="1">
-      <c r="B52" s="2" t="inlineStr">
+    <row r="56" ht="26" customHeight="1">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Wedding Command Center v1.0  ·  Edit Settings → Wedding Date · Budget · Guests  ·  Hyperlink nav chips to each sheet in Excel/Sheets</t>
         </is>
@@ -2205,7 +2205,7 @@
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B52:K52"/>
+    <mergeCell ref="B56:K56"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="B11:K11"/>
@@ -2321,10 +2321,10 @@
         </is>
       </c>
       <c r="D5" s="19" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>46136</v>
+        <v>46137</v>
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         </is>
       </c>
       <c r="D6" s="22" t="n">
-        <v>46161</v>
+        <v>46162</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>46156</v>
+        <v>46157</v>
       </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
@@ -2383,10 +2383,10 @@
         </is>
       </c>
       <c r="D7" s="19" t="n">
-        <v>46163</v>
+        <v>46164</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>46159</v>
+        <v>46160</v>
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
@@ -2413,7 +2413,7 @@
       </c>
       <c r="D8" s="22" t="n"/>
       <c r="E8" s="22" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="F8" s="21" t="inlineStr">
         <is>
@@ -2443,10 +2443,10 @@
         </is>
       </c>
       <c r="D9" s="19" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>46166</v>
+        <v>46167</v>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
@@ -2476,10 +2476,10 @@
         </is>
       </c>
       <c r="D10" s="22" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
       </c>
       <c r="D11" s="19" t="n"/>
       <c r="E11" s="19" t="n">
-        <v>46215</v>
+        <v>46216</v>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
@@ -2536,10 +2536,10 @@
         </is>
       </c>
       <c r="D12" s="22" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>46176</v>
+        <v>46177</v>
       </c>
       <c r="F12" s="21" t="inlineStr">
         <is>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="D13" s="19" t="n"/>
       <c r="E13" s="19" t="n">
-        <v>46208</v>
+        <v>46209</v>
       </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="F5" s="19" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
@@ -8660,7 +8660,7 @@
         </is>
       </c>
       <c r="F6" s="22" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
@@ -8755,7 +8755,7 @@
         </is>
       </c>
       <c r="F9" s="19" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="F10" s="22" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="G10" s="21" t="inlineStr">
         <is>
@@ -9109,7 +9109,7 @@
         </is>
       </c>
       <c r="C5" s="19" t="n">
-        <v>46171</v>
+        <v>46172</v>
       </c>
       <c r="D5" s="32" t="n">
         <v>120</v>
@@ -9137,7 +9137,7 @@
         </is>
       </c>
       <c r="C6" s="22" t="n">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D6" s="34" t="n">
         <v>180</v>
@@ -9165,7 +9165,7 @@
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="D7" s="32" t="n">
         <v>200</v>
@@ -9193,7 +9193,7 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>45</v>
@@ -9221,7 +9221,7 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="D9" s="32" t="n">
         <v>60</v>
@@ -9249,7 +9249,7 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>45</v>
@@ -9277,7 +9277,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="D11" s="32" t="n">
         <v>350</v>
@@ -9305,7 +9305,7 @@
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="D12" s="34" t="n">
         <v>220</v>
@@ -13091,7 +13091,7 @@
         </is>
       </c>
       <c r="C6" s="22" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D6" s="34" t="n">
         <v>2400</v>
@@ -13119,7 +13119,7 @@
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D7" s="32" t="n">
         <v>4200</v>
@@ -13147,7 +13147,7 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>46261</v>
+        <v>46262</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>180</v>
@@ -13171,7 +13171,7 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="D9" s="32" t="n">
         <v>350</v>
@@ -13199,7 +13199,7 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="D10" s="34" t="n">
         <v>200</v>
@@ -13223,7 +13223,7 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="D11" s="32" t="n">
         <v>160</v>
@@ -13247,7 +13247,7 @@
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="D12" s="34" t="n">
         <v>250</v>
@@ -13301,7 +13301,7 @@
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>46256</v>
+        <v>46257</v>
       </c>
       <c r="D14" s="34" t="n">
         <v>220</v>
@@ -14144,7 +14144,7 @@
         <v>450</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="E5" s="17" t="inlineStr">
         <is>
@@ -14172,7 +14172,7 @@
         <v>500</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
@@ -14196,7 +14196,7 @@
         <v>120</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="E7" s="17" t="inlineStr">
         <is>
@@ -14220,7 +14220,7 @@
         <v>700</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
@@ -14244,7 +14244,7 @@
         <v>100</v>
       </c>
       <c r="D9" s="19" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
@@ -14268,7 +14268,7 @@
         <v>60</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
@@ -14893,7 +14893,7 @@
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>46200</v>
+        <v>46201</v>
       </c>
       <c r="F8" s="21" t="inlineStr">
         <is>
@@ -14947,7 +14947,7 @@
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="F10" s="21" t="inlineStr"/>
     </row>
@@ -19595,7 +19595,7 @@
         </is>
       </c>
       <c r="E5" s="19" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
@@ -19630,7 +19630,7 @@
         </is>
       </c>
       <c r="E6" s="22" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
@@ -19665,7 +19665,7 @@
         </is>
       </c>
       <c r="E7" s="19" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
@@ -19700,7 +19700,7 @@
         </is>
       </c>
       <c r="E8" s="22" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
@@ -19735,7 +19735,7 @@
         </is>
       </c>
       <c r="E9" s="19" t="n">
-        <v>46181</v>
+        <v>46182</v>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
@@ -19770,7 +19770,7 @@
         </is>
       </c>
       <c r="E10" s="22" t="n">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
@@ -19805,7 +19805,7 @@
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>46226</v>
+        <v>46227</v>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
@@ -19840,7 +19840,7 @@
         </is>
       </c>
       <c r="E12" s="22" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
@@ -19875,7 +19875,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
@@ -19910,7 +19910,7 @@
         </is>
       </c>
       <c r="E14" s="22" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
@@ -19945,7 +19945,7 @@
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>46239</v>
+        <v>46240</v>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
@@ -19980,7 +19980,7 @@
         </is>
       </c>
       <c r="E16" s="22" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
@@ -20015,7 +20015,7 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
@@ -20050,7 +20050,7 @@
         </is>
       </c>
       <c r="E18" s="22" t="n">
-        <v>46223</v>
+        <v>46224</v>
       </c>
       <c r="F18" s="20" t="inlineStr">
         <is>
@@ -20085,7 +20085,7 @@
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
@@ -20120,7 +20120,7 @@
         </is>
       </c>
       <c r="E20" s="22" t="n">
-        <v>46243</v>
+        <v>46244</v>
       </c>
       <c r="F20" s="20" t="inlineStr">
         <is>
@@ -20155,7 +20155,7 @@
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
@@ -20190,7 +20190,7 @@
         </is>
       </c>
       <c r="E22" s="22" t="n">
-        <v>46244</v>
+        <v>46245</v>
       </c>
       <c r="F22" s="20" t="inlineStr">
         <is>
@@ -22342,7 +22342,7 @@
         <v>6000</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
@@ -22380,7 +22380,7 @@
         <v>3000</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>46246</v>
+        <v>46247</v>
       </c>
       <c r="F6" s="20" t="inlineStr">
         <is>
@@ -22418,7 +22418,7 @@
         <v>2000</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>46251</v>
+        <v>46252</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
@@ -22456,7 +22456,7 @@
         <v>2300</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>46221</v>
+        <v>46222</v>
       </c>
       <c r="F8" s="20" t="inlineStr">
         <is>
@@ -22494,7 +22494,7 @@
         <v>650</v>
       </c>
       <c r="E9" s="19" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
@@ -22532,7 +22532,7 @@
         <v>7000</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>46241</v>
+        <v>46242</v>
       </c>
       <c r="F10" s="20" t="inlineStr">
         <is>
@@ -22570,7 +22570,7 @@
         <v>1700</v>
       </c>
       <c r="E11" s="19" t="n">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
@@ -22608,7 +22608,7 @@
         <v>1500</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="F12" s="20" t="inlineStr">
         <is>
@@ -22646,7 +22646,7 @@
         <v>1400</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>46216</v>
+        <v>46217</v>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
@@ -22684,7 +22684,7 @@
         <v>800</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>

</xml_diff>